<commit_message>
BS-02: EXAMPLE fixture uses listed NZX codes (FPH.NZ, AIR.NZ) so the symbol check passes
</commit_message>
<xml_diff>
--- a/src/lib/fixtures/broker-import/investnow/investnow-example-bad-rows.xlsx
+++ b/src/lib/fixtures/broker-import/investnow/investnow-example-bad-rows.xlsx
@@ -443,7 +443,7 @@
         <v>2025-05-02</v>
       </c>
       <c r="B5" t="str">
-        <v>FNZ.NZ</v>
+        <v>FPH.NZ</v>
       </c>
       <c r="C5" t="str">
         <v>Buy</v>
@@ -501,7 +501,7 @@
         <v>2025-08-15</v>
       </c>
       <c r="B7" t="str">
-        <v>FNZ.NZ</v>
+        <v>FPH.NZ</v>
       </c>
       <c r="C7" t="str">
         <v>Sell</v>
@@ -530,7 +530,7 @@
         <v>2025-09-01</v>
       </c>
       <c r="B8" t="str">
-        <v>USF.NZ</v>
+        <v>AIR.NZ</v>
       </c>
       <c r="C8" t="str">
         <v>Buy</v>
@@ -559,7 +559,7 @@
         <v>not-a-date</v>
       </c>
       <c r="B9" t="str">
-        <v>FNZ.NZ</v>
+        <v>FPH.NZ</v>
       </c>
       <c r="C9" t="str">
         <v>Buy</v>
@@ -588,7 +588,7 @@
         <v>2025-10-01</v>
       </c>
       <c r="B10" t="str">
-        <v>USF.NZ</v>
+        <v>AIR.NZ</v>
       </c>
       <c r="C10" t="str">
         <v>Buy</v>

</xml_diff>